<commit_message>
تحديث جديد Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/saved_files/shipments_data.xlsx
+++ b/saved_files/shipments_data.xlsx
@@ -7,11 +7,11 @@
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Sheet1!$A$1:$L$1035</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_0BCC3106_3BC2_4BD7_A8C5_60E33E565406_.wvu.FilterData">Sheet1!$A$1:$L$1035</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_49F3F851_3D4E_4D67_A629_29765EB87497_.wvu.FilterData">Sheet1!$A$1:$L$1035</definedName>
   </definedNames>
   <calcPr/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{0BCC3106-3BC2-4BD7-A8C5-60E33E565406}" name="Table1 filter view"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{49F3F851-3D4E-4D67-A629-29765EB87497}" name="Table1 filter view"/>
   </customWorkbookViews>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
@@ -165,28 +165,19 @@
     <t>B12</t>
   </si>
   <si>
-    <t>B6609</t>
-  </si>
-  <si>
     <t>B1984</t>
   </si>
   <si>
     <t>B44</t>
   </si>
   <si>
-    <t>DH132</t>
+    <t>B4719</t>
+  </si>
+  <si>
+    <t>B5709</t>
   </si>
   <si>
     <t>مخزن أربيل</t>
-  </si>
-  <si>
-    <t>B4719</t>
-  </si>
-  <si>
-    <t>E161</t>
-  </si>
-  <si>
-    <t>B5709</t>
   </si>
   <si>
     <t>B5772</t>
@@ -195,10 +186,7 @@
     <t>B6224</t>
   </si>
   <si>
-    <t>M442</t>
-  </si>
-  <si>
-    <t>M685</t>
+    <t>B6609</t>
   </si>
   <si>
     <t>B7148</t>
@@ -216,6 +204,12 @@
     <t>BS3428</t>
   </si>
   <si>
+    <t>DH132</t>
+  </si>
+  <si>
+    <t>E161</t>
+  </si>
+  <si>
     <t>H71</t>
   </si>
   <si>
@@ -223,6 +217,12 @@
   </si>
   <si>
     <t>KB501</t>
+  </si>
+  <si>
+    <t>M442</t>
+  </si>
+  <si>
+    <t>M685</t>
   </si>
   <si>
     <t>SM172</t>
@@ -239,7 +239,7 @@
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="18.0"/>
       <color theme="1"/>
@@ -253,6 +253,16 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b/>
       <sz val="24.0"/>
       <color rgb="FF000000"/>
@@ -264,7 +274,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,6 +287,18 @@
         <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8CDDFA"/>
+        <bgColor rgb="FF8CDDFA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -284,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -321,31 +343,43 @@
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -716,7 +750,7 @@
         <v>6.5</v>
       </c>
       <c r="G2" s="9">
-        <f t="shared" ref="G2:G60" si="1">C2*F2</f>
+        <f t="shared" ref="G2:G35" si="1">C2*F2</f>
         <v>1755</v>
       </c>
       <c r="H2" s="10"/>
@@ -2298,29 +2332,28 @@
       <c r="A36" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="13">
         <v>41.9</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="13">
         <v>1.0</v>
       </c>
-      <c r="E36" s="12">
+      <c r="E36" s="13">
         <v>0.181</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="14">
         <v>6.5</v>
       </c>
-      <c r="G36" s="9">
-        <f t="shared" si="1"/>
+      <c r="G36" s="15">
         <v>272.35</v>
       </c>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="14" t="s">
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="17" t="s">
         <v>44</v>
       </c>
       <c r="L36" s="11" t="s">
@@ -2345,29 +2378,28 @@
       <c r="A37" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="13">
         <v>712.5</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="13">
         <v>17.0</v>
       </c>
-      <c r="E37" s="12">
+      <c r="E37" s="13">
         <v>2.63</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="14">
         <v>6.5</v>
       </c>
-      <c r="G37" s="9">
-        <f t="shared" si="1"/>
+      <c r="G37" s="15">
         <v>4631.25</v>
       </c>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="13"/>
-      <c r="K37" s="14" t="s">
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="17" t="s">
         <v>44</v>
       </c>
       <c r="L37" s="11" t="s">
@@ -2392,29 +2424,28 @@
       <c r="A38" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C38" s="15">
+      <c r="C38" s="18">
         <v>2221.8</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="13">
         <v>48.0</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="13">
         <v>10.477</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="14">
         <v>6.5</v>
       </c>
-      <c r="G38" s="9">
-        <f t="shared" si="1"/>
+      <c r="G38" s="15">
         <v>14441.7</v>
       </c>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="13"/>
-      <c r="K38" s="14" t="s">
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="17" t="s">
         <v>44</v>
       </c>
       <c r="L38" s="11" t="s">
@@ -2439,29 +2470,28 @@
       <c r="A39" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="12">
-        <v>1303.5</v>
-      </c>
-      <c r="D39" s="12">
-        <v>25.0</v>
-      </c>
-      <c r="E39" s="12">
-        <v>4.415</v>
-      </c>
-      <c r="F39" s="8">
+      <c r="C39" s="13">
+        <v>514.7</v>
+      </c>
+      <c r="D39" s="13">
+        <v>17.0</v>
+      </c>
+      <c r="E39" s="13">
+        <v>2.063</v>
+      </c>
+      <c r="F39" s="14">
         <v>6.5</v>
       </c>
-      <c r="G39" s="9">
-        <f t="shared" si="1"/>
-        <v>8472.75</v>
-      </c>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="14" t="s">
+      <c r="G39" s="15">
+        <v>3345.55</v>
+      </c>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="17" t="s">
         <v>44</v>
       </c>
       <c r="L39" s="11" t="s">
@@ -2486,32 +2516,31 @@
       <c r="A40" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C40" s="12">
-        <v>514.7</v>
-      </c>
-      <c r="D40" s="12">
-        <v>17.0</v>
-      </c>
-      <c r="E40" s="12">
-        <v>2.063</v>
-      </c>
-      <c r="F40" s="8">
+      <c r="C40" s="13">
+        <v>92.1</v>
+      </c>
+      <c r="D40" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="E40" s="13">
+        <v>0.431</v>
+      </c>
+      <c r="F40" s="14">
         <v>6.5</v>
       </c>
-      <c r="G40" s="9">
-        <f t="shared" si="1"/>
-        <v>3345.55</v>
-      </c>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
-      <c r="J40" s="13"/>
-      <c r="K40" s="14" t="s">
+      <c r="G40" s="15">
+        <v>598.65</v>
+      </c>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L40" s="14" t="s">
+      <c r="L40" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M40" s="6"/>
@@ -2533,32 +2562,31 @@
       <c r="A41" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C41" s="12">
-        <v>92.1</v>
-      </c>
-      <c r="D41" s="12">
+      <c r="B41" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="13">
+        <v>141.4</v>
+      </c>
+      <c r="D41" s="13">
         <v>3.0</v>
       </c>
-      <c r="E41" s="12">
-        <v>0.431</v>
-      </c>
-      <c r="F41" s="8">
+      <c r="E41" s="13">
+        <v>0.485</v>
+      </c>
+      <c r="F41" s="14">
         <v>6.5</v>
       </c>
-      <c r="G41" s="9">
-        <f t="shared" si="1"/>
-        <v>598.65</v>
-      </c>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="14" t="s">
+      <c r="G41" s="15">
+        <v>919.1</v>
+      </c>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L41" s="14" t="s">
+      <c r="L41" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M41" s="6"/>
@@ -2580,32 +2608,31 @@
       <c r="A42" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C42" s="12">
-        <v>141.4</v>
-      </c>
-      <c r="D42" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="E42" s="12">
-        <v>0.485</v>
-      </c>
-      <c r="F42" s="8">
+      <c r="B42" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C42" s="13">
+        <v>95.4</v>
+      </c>
+      <c r="D42" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="E42" s="13">
+        <v>0.482</v>
+      </c>
+      <c r="F42" s="14">
         <v>6.5</v>
       </c>
-      <c r="G42" s="9">
-        <f t="shared" si="1"/>
-        <v>919.1</v>
-      </c>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
-      <c r="J42" s="13"/>
-      <c r="K42" s="14" t="s">
+      <c r="G42" s="15">
+        <v>620.1</v>
+      </c>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+      <c r="J42" s="16"/>
+      <c r="K42" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L42" s="14" t="s">
+      <c r="L42" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M42" s="6"/>
@@ -2627,32 +2654,31 @@
       <c r="A43" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C43" s="12">
-        <v>32.8</v>
-      </c>
-      <c r="D43" s="12">
-        <v>2.0</v>
-      </c>
-      <c r="E43" s="12">
-        <v>0.143</v>
-      </c>
-      <c r="F43" s="8">
+      <c r="C43" s="13">
+        <v>792.5</v>
+      </c>
+      <c r="D43" s="13">
+        <v>17.0</v>
+      </c>
+      <c r="E43" s="13">
+        <v>3.002</v>
+      </c>
+      <c r="F43" s="14">
         <v>6.5</v>
       </c>
-      <c r="G43" s="9">
-        <f t="shared" si="1"/>
-        <v>213.2</v>
-      </c>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
-      <c r="J43" s="13"/>
-      <c r="K43" s="14" t="s">
+      <c r="G43" s="15">
+        <v>5151.25</v>
+      </c>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+      <c r="J43" s="16"/>
+      <c r="K43" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L43" s="14" t="s">
+      <c r="L43" s="17" t="s">
         <v>51</v>
       </c>
       <c r="M43" s="6"/>
@@ -2674,32 +2700,31 @@
       <c r="A44" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C44" s="15">
-        <v>95.4</v>
-      </c>
-      <c r="D44" s="12">
-        <v>5.0</v>
-      </c>
-      <c r="E44" s="12">
-        <v>0.482</v>
-      </c>
-      <c r="F44" s="8">
+      <c r="C44" s="18">
+        <v>2521.6</v>
+      </c>
+      <c r="D44" s="13">
+        <v>111.0</v>
+      </c>
+      <c r="E44" s="13">
+        <v>12.252</v>
+      </c>
+      <c r="F44" s="14">
         <v>6.5</v>
       </c>
-      <c r="G44" s="9">
-        <f t="shared" si="1"/>
-        <v>620.1</v>
-      </c>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
-      <c r="J44" s="13"/>
-      <c r="K44" s="14" t="s">
+      <c r="G44" s="15">
+        <v>16390.4</v>
+      </c>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L44" s="14" t="s">
+      <c r="L44" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M44" s="6"/>
@@ -2721,32 +2746,31 @@
       <c r="A45" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C45" s="12">
-        <v>425.5</v>
-      </c>
-      <c r="D45" s="12">
-        <v>8.0</v>
-      </c>
-      <c r="E45" s="12">
-        <v>1.988</v>
-      </c>
-      <c r="F45" s="8">
+      <c r="C45" s="13">
+        <v>55.1</v>
+      </c>
+      <c r="D45" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="E45" s="13">
+        <v>0.247</v>
+      </c>
+      <c r="F45" s="14">
         <v>6.5</v>
       </c>
-      <c r="G45" s="9">
-        <f t="shared" si="1"/>
-        <v>2765.75</v>
-      </c>
-      <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
-      <c r="J45" s="13"/>
-      <c r="K45" s="14" t="s">
+      <c r="G45" s="15">
+        <v>358.15</v>
+      </c>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L45" s="14" t="s">
+      <c r="L45" s="17" t="s">
         <v>51</v>
       </c>
       <c r="M45" s="6"/>
@@ -2768,32 +2792,31 @@
       <c r="A46" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C46" s="15">
-        <v>792.5</v>
-      </c>
-      <c r="D46" s="12">
-        <v>17.0</v>
-      </c>
-      <c r="E46" s="12">
-        <v>3.002</v>
-      </c>
-      <c r="F46" s="8">
+      <c r="C46" s="18">
+        <v>1303.5</v>
+      </c>
+      <c r="D46" s="13">
+        <v>25.0</v>
+      </c>
+      <c r="E46" s="13">
+        <v>4.415</v>
+      </c>
+      <c r="F46" s="14">
         <v>6.5</v>
       </c>
-      <c r="G46" s="9">
-        <f t="shared" si="1"/>
-        <v>5151.25</v>
-      </c>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
-      <c r="J46" s="13"/>
-      <c r="K46" s="14" t="s">
+      <c r="G46" s="15">
+        <v>8472.75</v>
+      </c>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L46" s="14" t="s">
+      <c r="L46" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M46" s="6"/>
@@ -2815,32 +2838,31 @@
       <c r="A47" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B47" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C47" s="12">
-        <v>2521.6</v>
-      </c>
-      <c r="D47" s="12">
-        <v>111.0</v>
-      </c>
-      <c r="E47" s="12">
-        <v>12.252</v>
-      </c>
-      <c r="F47" s="8">
+      <c r="C47" s="13">
+        <v>18.1</v>
+      </c>
+      <c r="D47" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="E47" s="13">
+        <v>0.099</v>
+      </c>
+      <c r="F47" s="14">
         <v>6.5</v>
       </c>
-      <c r="G47" s="9">
-        <f t="shared" si="1"/>
-        <v>16390.4</v>
-      </c>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
-      <c r="J47" s="13"/>
-      <c r="K47" s="14" t="s">
+      <c r="G47" s="15">
+        <v>117.65</v>
+      </c>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L47" s="14" t="s">
+      <c r="L47" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M47" s="6"/>
@@ -2862,32 +2884,31 @@
       <c r="A48" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C48" s="12">
-        <v>55.1</v>
-      </c>
-      <c r="D48" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="E48" s="12">
-        <v>0.247</v>
-      </c>
-      <c r="F48" s="8">
+      <c r="C48" s="13">
+        <v>86.9</v>
+      </c>
+      <c r="D48" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="E48" s="13">
+        <v>0.787</v>
+      </c>
+      <c r="F48" s="14">
         <v>6.5</v>
       </c>
-      <c r="G48" s="9">
-        <f t="shared" si="1"/>
-        <v>358.15</v>
-      </c>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="13"/>
-      <c r="K48" s="14" t="s">
+      <c r="G48" s="15">
+        <v>564.85</v>
+      </c>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16"/>
+      <c r="J48" s="16"/>
+      <c r="K48" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L48" s="14" t="s">
+      <c r="L48" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M48" s="6"/>
@@ -2909,32 +2930,31 @@
       <c r="A49" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="B49" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C49" s="12">
-        <v>156.3</v>
-      </c>
-      <c r="D49" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="E49" s="12">
-        <v>0.852</v>
-      </c>
-      <c r="F49" s="8">
+      <c r="C49" s="13">
+        <v>802.9</v>
+      </c>
+      <c r="D49" s="13">
+        <v>30.0</v>
+      </c>
+      <c r="E49" s="13">
+        <v>3.923</v>
+      </c>
+      <c r="F49" s="14">
         <v>6.5</v>
       </c>
-      <c r="G49" s="9">
-        <f t="shared" si="1"/>
-        <v>1015.95</v>
-      </c>
-      <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
-      <c r="J49" s="13"/>
-      <c r="K49" s="14" t="s">
+      <c r="G49" s="15">
+        <v>5218.85</v>
+      </c>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16"/>
+      <c r="J49" s="16"/>
+      <c r="K49" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L49" s="14" t="s">
+      <c r="L49" s="17" t="s">
         <v>15</v>
       </c>
       <c r="M49" s="6"/>
@@ -2956,32 +2976,31 @@
       <c r="A50" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="12">
-        <v>431.5</v>
-      </c>
-      <c r="D50" s="12">
-        <v>17.0</v>
-      </c>
-      <c r="E50" s="12">
-        <v>1.991</v>
-      </c>
-      <c r="F50" s="8">
+      <c r="C50" s="13">
+        <v>229.0</v>
+      </c>
+      <c r="D50" s="13">
+        <v>18.0</v>
+      </c>
+      <c r="E50" s="13">
+        <v>2.14</v>
+      </c>
+      <c r="F50" s="14">
         <v>6.5</v>
       </c>
-      <c r="G50" s="9">
-        <f t="shared" si="1"/>
-        <v>2804.75</v>
-      </c>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
-      <c r="J50" s="13"/>
-      <c r="K50" s="14" t="s">
+      <c r="G50" s="15">
+        <v>1488.5</v>
+      </c>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16"/>
+      <c r="J50" s="16"/>
+      <c r="K50" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L50" s="14" t="s">
+      <c r="L50" s="17" t="s">
         <v>15</v>
       </c>
       <c r="M50" s="6"/>
@@ -3003,32 +3022,31 @@
       <c r="A51" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C51" s="12">
-        <v>18.1</v>
-      </c>
-      <c r="D51" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="E51" s="12">
-        <v>0.099</v>
-      </c>
-      <c r="F51" s="8">
-        <v>6.5</v>
-      </c>
-      <c r="G51" s="9">
-        <f t="shared" si="1"/>
-        <v>117.65</v>
-      </c>
-      <c r="H51" s="13"/>
-      <c r="I51" s="13"/>
-      <c r="J51" s="13"/>
-      <c r="K51" s="14" t="s">
+      <c r="C51" s="13">
+        <v>190.0</v>
+      </c>
+      <c r="D51" s="13">
+        <v>20.0</v>
+      </c>
+      <c r="E51" s="13">
+        <v>1.495</v>
+      </c>
+      <c r="F51" s="19">
+        <v>7.0</v>
+      </c>
+      <c r="G51" s="15">
+        <v>1330.0</v>
+      </c>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16"/>
+      <c r="J51" s="16"/>
+      <c r="K51" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L51" s="14" t="s">
+      <c r="L51" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M51" s="6"/>
@@ -3050,32 +3068,31 @@
       <c r="A52" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B52" s="12" t="s">
+      <c r="B52" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C52" s="12">
-        <v>86.9</v>
-      </c>
-      <c r="D52" s="12">
-        <v>4.0</v>
-      </c>
-      <c r="E52" s="12">
-        <v>0.787</v>
-      </c>
-      <c r="F52" s="8">
+      <c r="C52" s="13">
+        <v>32.8</v>
+      </c>
+      <c r="D52" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="E52" s="13">
+        <v>0.143</v>
+      </c>
+      <c r="F52" s="14">
         <v>6.5</v>
       </c>
-      <c r="G52" s="9">
-        <f t="shared" si="1"/>
-        <v>564.85</v>
-      </c>
-      <c r="H52" s="13"/>
-      <c r="I52" s="13"/>
-      <c r="J52" s="13"/>
-      <c r="K52" s="14" t="s">
+      <c r="G52" s="15">
+        <v>213.2</v>
+      </c>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L52" s="14" t="s">
+      <c r="L52" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M52" s="6"/>
@@ -3097,32 +3114,31 @@
       <c r="A53" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B53" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="C53" s="12">
-        <v>802.9</v>
-      </c>
-      <c r="D53" s="12">
-        <v>30.0</v>
-      </c>
-      <c r="E53" s="12">
-        <v>3.923</v>
-      </c>
-      <c r="F53" s="8">
+      <c r="B53" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" s="13">
+        <v>201.3</v>
+      </c>
+      <c r="D53" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="E53" s="13">
+        <v>1.008</v>
+      </c>
+      <c r="F53" s="14">
         <v>6.5</v>
       </c>
-      <c r="G53" s="9">
-        <f t="shared" si="1"/>
-        <v>5218.85</v>
-      </c>
-      <c r="H53" s="13"/>
-      <c r="I53" s="13"/>
-      <c r="J53" s="13"/>
-      <c r="K53" s="14" t="s">
+      <c r="G53" s="15">
+        <v>1308.45</v>
+      </c>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16"/>
+      <c r="J53" s="16"/>
+      <c r="K53" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L53" s="14" t="s">
+      <c r="L53" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M53" s="6"/>
@@ -3144,32 +3160,31 @@
       <c r="A54" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B54" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="C54" s="12">
-        <v>229.0</v>
-      </c>
-      <c r="D54" s="12">
-        <v>18.0</v>
-      </c>
-      <c r="E54" s="12">
-        <v>2.14</v>
-      </c>
-      <c r="F54" s="8">
+      <c r="B54" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C54" s="13">
+        <v>425.5</v>
+      </c>
+      <c r="D54" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="E54" s="13">
+        <v>1.988</v>
+      </c>
+      <c r="F54" s="14">
         <v>6.5</v>
       </c>
-      <c r="G54" s="9">
-        <f t="shared" si="1"/>
-        <v>1488.5</v>
-      </c>
-      <c r="H54" s="13"/>
-      <c r="I54" s="13"/>
-      <c r="J54" s="13"/>
-      <c r="K54" s="14" t="s">
+      <c r="G54" s="15">
+        <v>2765.75</v>
+      </c>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16"/>
+      <c r="J54" s="16"/>
+      <c r="K54" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L54" s="14" t="s">
+      <c r="L54" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M54" s="6"/>
@@ -3191,32 +3206,31 @@
       <c r="A55" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B55" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C55" s="12">
-        <v>190.0</v>
-      </c>
-      <c r="D55" s="12">
-        <v>20.0</v>
-      </c>
-      <c r="E55" s="12">
-        <v>1.495</v>
-      </c>
-      <c r="F55" s="8">
+      <c r="B55" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C55" s="13">
+        <v>287.3</v>
+      </c>
+      <c r="D55" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="E55" s="13">
+        <v>1.883</v>
+      </c>
+      <c r="F55" s="14">
         <v>6.5</v>
       </c>
-      <c r="G55" s="9">
-        <f t="shared" si="1"/>
-        <v>1235</v>
-      </c>
-      <c r="H55" s="13"/>
-      <c r="I55" s="13"/>
-      <c r="J55" s="13"/>
-      <c r="K55" s="14" t="s">
+      <c r="G55" s="15">
+        <v>1867.45</v>
+      </c>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
+      <c r="J55" s="16"/>
+      <c r="K55" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L55" s="14" t="s">
+      <c r="L55" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M55" s="6"/>
@@ -3238,32 +3252,31 @@
       <c r="A56" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B56" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C56" s="12">
-        <v>201.3</v>
-      </c>
-      <c r="D56" s="12">
-        <v>5.0</v>
-      </c>
-      <c r="E56" s="12">
-        <v>1.008</v>
-      </c>
-      <c r="F56" s="8">
+      <c r="B56" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C56" s="13">
+        <v>141.4</v>
+      </c>
+      <c r="D56" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="E56" s="13">
+        <v>0.754</v>
+      </c>
+      <c r="F56" s="14">
         <v>6.5</v>
       </c>
-      <c r="G56" s="9">
-        <f t="shared" si="1"/>
-        <v>1308.45</v>
-      </c>
-      <c r="H56" s="13"/>
-      <c r="I56" s="13"/>
-      <c r="J56" s="13"/>
-      <c r="K56" s="14" t="s">
+      <c r="G56" s="15">
+        <v>919.1</v>
+      </c>
+      <c r="H56" s="16"/>
+      <c r="I56" s="16"/>
+      <c r="J56" s="16"/>
+      <c r="K56" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L56" s="14" t="s">
+      <c r="L56" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M56" s="6"/>
@@ -3285,32 +3298,31 @@
       <c r="A57" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C57" s="12">
-        <v>287.3</v>
-      </c>
-      <c r="D57" s="12">
+      <c r="C57" s="13">
+        <v>644.4</v>
+      </c>
+      <c r="D57" s="13">
+        <v>24.0</v>
+      </c>
+      <c r="E57" s="13">
+        <v>3.159</v>
+      </c>
+      <c r="F57" s="19">
         <v>8.0</v>
       </c>
-      <c r="E57" s="12">
-        <v>1.883</v>
-      </c>
-      <c r="F57" s="8">
-        <v>6.5</v>
-      </c>
-      <c r="G57" s="9">
-        <f t="shared" si="1"/>
-        <v>1867.45</v>
-      </c>
-      <c r="H57" s="13"/>
-      <c r="I57" s="13"/>
-      <c r="J57" s="13"/>
-      <c r="K57" s="14" t="s">
+      <c r="G57" s="15">
+        <v>5155.2</v>
+      </c>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
+      <c r="J57" s="16"/>
+      <c r="K57" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L57" s="14" t="s">
+      <c r="L57" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M57" s="6"/>
@@ -3332,32 +3344,31 @@
       <c r="A58" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C58" s="12">
-        <v>141.4</v>
-      </c>
-      <c r="D58" s="12">
+      <c r="C58" s="13">
+        <v>156.3</v>
+      </c>
+      <c r="D58" s="13">
         <v>3.0</v>
       </c>
-      <c r="E58" s="12">
-        <v>0.754</v>
-      </c>
-      <c r="F58" s="8">
+      <c r="E58" s="13">
+        <v>0.852</v>
+      </c>
+      <c r="F58" s="14">
         <v>6.5</v>
       </c>
-      <c r="G58" s="9">
-        <f t="shared" si="1"/>
-        <v>919.1</v>
-      </c>
-      <c r="H58" s="13"/>
-      <c r="I58" s="13"/>
-      <c r="J58" s="13"/>
-      <c r="K58" s="14" t="s">
+      <c r="G58" s="15">
+        <v>1015.95</v>
+      </c>
+      <c r="H58" s="16"/>
+      <c r="I58" s="16"/>
+      <c r="J58" s="16"/>
+      <c r="K58" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L58" s="14" t="s">
+      <c r="L58" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M58" s="6"/>
@@ -3379,32 +3390,31 @@
       <c r="A59" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C59" s="12">
-        <v>644.4</v>
-      </c>
-      <c r="D59" s="12">
-        <v>24.0</v>
-      </c>
-      <c r="E59" s="12">
-        <v>3.159</v>
-      </c>
-      <c r="F59" s="8">
+      <c r="C59" s="13">
+        <v>431.5</v>
+      </c>
+      <c r="D59" s="13">
+        <v>17.0</v>
+      </c>
+      <c r="E59" s="13">
+        <v>1.991</v>
+      </c>
+      <c r="F59" s="14">
         <v>6.5</v>
       </c>
-      <c r="G59" s="9">
-        <f t="shared" si="1"/>
-        <v>4188.6</v>
-      </c>
-      <c r="H59" s="13"/>
-      <c r="I59" s="13"/>
-      <c r="J59" s="13"/>
-      <c r="K59" s="14" t="s">
+      <c r="G59" s="15">
+        <v>2804.75</v>
+      </c>
+      <c r="H59" s="16"/>
+      <c r="I59" s="16"/>
+      <c r="J59" s="16"/>
+      <c r="K59" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L59" s="14" t="s">
+      <c r="L59" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M59" s="6"/>
@@ -3426,32 +3436,31 @@
       <c r="A60" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B60" s="12" t="s">
+      <c r="B60" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C60" s="12">
+      <c r="C60" s="13">
         <v>117.3</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="13">
         <v>6.0</v>
       </c>
-      <c r="E60" s="12">
+      <c r="E60" s="13">
         <v>0.523</v>
       </c>
-      <c r="F60" s="8">
+      <c r="F60" s="14">
         <v>6.5</v>
       </c>
-      <c r="G60" s="9">
-        <f t="shared" si="1"/>
+      <c r="G60" s="15">
         <v>762.45</v>
       </c>
-      <c r="H60" s="13"/>
-      <c r="I60" s="13"/>
-      <c r="J60" s="13"/>
-      <c r="K60" s="14" t="s">
+      <c r="H60" s="16"/>
+      <c r="I60" s="16"/>
+      <c r="J60" s="16"/>
+      <c r="K60" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L60" s="14" t="s">
+      <c r="L60" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M60" s="6"/>
@@ -3470,35 +3479,35 @@
       <c r="Z60" s="6"/>
     </row>
     <row r="61" ht="28.5" customHeight="1">
-      <c r="A61" s="16" t="s">
+      <c r="A61" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C61" s="17">
+      <c r="C61" s="21">
         <v>16426.0</v>
       </c>
-      <c r="D61" s="17">
+      <c r="D61" s="21">
         <v>668.0</v>
       </c>
-      <c r="E61" s="17">
+      <c r="E61" s="21">
         <v>68.649</v>
       </c>
       <c r="F61" s="8">
         <v>325.0</v>
       </c>
-      <c r="G61" s="18">
+      <c r="G61" s="22">
         <f>E61*F61</f>
         <v>22310.925</v>
       </c>
-      <c r="H61" s="19"/>
-      <c r="I61" s="19"/>
-      <c r="J61" s="19"/>
-      <c r="K61" s="20" t="s">
+      <c r="H61" s="23"/>
+      <c r="I61" s="23"/>
+      <c r="J61" s="23"/>
+      <c r="K61" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="L61" s="14" t="s">
+      <c r="L61" s="17" t="s">
         <v>19</v>
       </c>
       <c r="M61" s="6"/>
@@ -3517,18 +3526,18 @@
       <c r="Z61" s="6"/>
     </row>
     <row r="62" ht="28.5" customHeight="1">
-      <c r="A62" s="16"/>
-      <c r="B62" s="16"/>
-      <c r="C62" s="17"/>
-      <c r="D62" s="17"/>
-      <c r="E62" s="17"/>
+      <c r="A62" s="20"/>
+      <c r="B62" s="20"/>
+      <c r="C62" s="21"/>
+      <c r="D62" s="21"/>
+      <c r="E62" s="21"/>
       <c r="F62" s="8"/>
-      <c r="G62" s="18"/>
-      <c r="H62" s="19"/>
-      <c r="I62" s="19"/>
-      <c r="J62" s="19"/>
-      <c r="K62" s="20"/>
-      <c r="L62" s="14"/>
+      <c r="G62" s="22"/>
+      <c r="H62" s="23"/>
+      <c r="I62" s="23"/>
+      <c r="J62" s="23"/>
+      <c r="K62" s="24"/>
+      <c r="L62" s="17"/>
       <c r="M62" s="6"/>
       <c r="N62" s="6"/>
       <c r="O62" s="6"/>
@@ -30790,7 +30799,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{0BCC3106-3BC2-4BD7-A8C5-60E33E565406}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{49F3F851-3D4E-4D67-A629-29765EB87497}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$L$1035"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">

</xml_diff>